<commit_message>
Visual polish: sev-badge unificado, toggle fix, wow-pill, colwidths W21
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9395,7 +9395,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12359,7 +12359,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15605,7 +15605,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15758,7 +15758,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15911,7 +15911,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16071,7 +16071,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19505,7 +19505,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -23804,7 +23804,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28103,7 +28103,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -29761,7 +29761,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33355,7 +33355,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33774,7 +33774,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38067,7 +38067,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38227,7 +38227,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42825,7 +42825,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42985,7 +42985,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45069,7 +45069,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -49368,7 +49368,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -51441,7 +51441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52979,7 +52979,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56573,7 +56573,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56992,7 +56992,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -61291,7 +61291,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -65589,7 +65589,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -69583,7 +69583,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71441,7 +71441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75035,7 +75035,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75454,7 +75454,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 17:15 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix WoW RND: enriquecer TOP[] con p80_hotel para evitar NaN por duplicados en merge
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9395,7 +9395,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12359,7 +12359,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15605,7 +15605,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15758,7 +15758,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15911,7 +15911,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16071,7 +16071,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19505,7 +19505,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -23804,7 +23804,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28103,7 +28103,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -29761,7 +29761,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33355,7 +33355,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33774,7 +33774,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38067,7 +38067,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38227,7 +38227,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42825,7 +42825,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42985,7 +42985,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45069,7 +45069,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -49368,7 +49368,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -51441,7 +51441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52979,7 +52979,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56573,7 +56573,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56992,7 +56992,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -61291,7 +61291,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -65589,7 +65589,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -69583,7 +69583,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71441,7 +71441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75035,7 +75035,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75454,7 +75454,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 21:56 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix WoW CR: enriquecer TOP[] con TAB_EF/TAB_CV para evitar NaN en tabs hotel
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9395,7 +9395,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12359,7 +12359,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15605,7 +15605,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15758,7 +15758,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15911,7 +15911,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16071,7 +16071,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19505,7 +19505,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -23804,7 +23804,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28103,7 +28103,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -29761,7 +29761,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33355,7 +33355,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33774,7 +33774,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38067,7 +38067,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38227,7 +38227,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42825,7 +42825,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42985,7 +42985,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45069,7 +45069,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -49368,7 +49368,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -51441,7 +51441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52979,7 +52979,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56573,7 +56573,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56992,7 +56992,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -61291,7 +61291,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -65589,7 +65589,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -69583,7 +69583,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71441,7 +71441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75035,7 +75035,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75454,7 +75454,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:13 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix WoW canastas: enriquecer CANASTA[] sub-dfs con WoW desde p80_hotel/TAB_EF/TAB_CV
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9395,7 +9395,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12359,7 +12359,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15605,7 +15605,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15758,7 +15758,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15911,7 +15911,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16071,7 +16071,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19505,7 +19505,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -23804,7 +23804,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28103,7 +28103,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -29761,7 +29761,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33355,7 +33355,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33774,7 +33774,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38067,7 +38067,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38227,7 +38227,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42825,7 +42825,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42985,7 +42985,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45069,7 +45069,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -49368,7 +49368,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -51441,7 +51441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52979,7 +52979,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56573,7 +56573,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56992,7 +56992,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -61291,7 +61291,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -65589,7 +65589,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -69583,7 +69583,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71441,7 +71441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75035,7 +75035,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75454,7 +75454,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:21 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix CSS: tabs activos heredaban background de .canasta-block por selector sin cierre
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9395,7 +9395,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12359,7 +12359,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15605,7 +15605,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15758,7 +15758,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15911,7 +15911,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16071,7 +16071,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19505,7 +19505,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -23804,7 +23804,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28103,7 +28103,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -29761,7 +29761,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33355,7 +33355,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33774,7 +33774,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38067,7 +38067,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38227,7 +38227,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42825,7 +42825,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42985,7 +42985,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45069,7 +45069,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -49368,7 +49368,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -51441,7 +51441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52979,7 +52979,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56573,7 +56573,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56992,7 +56992,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -61291,7 +61291,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -65589,7 +65589,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -69583,7 +69583,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71441,7 +71441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75035,7 +75035,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75454,7 +75454,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 22:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 22:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel canastas: top100 desde p80, orden %NoDispo DESC / Eficacia ASC, formato 0.00%, limpieza ID hotel
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9395,7 +9395,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12359,7 +12359,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12698,7 +12698,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15605,7 +15605,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15758,7 +15758,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -15911,7 +15911,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16071,7 +16071,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19505,7 +19505,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -23804,7 +23804,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28103,7 +28103,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -29761,7 +29761,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33355,7 +33355,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -33774,7 +33774,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38067,7 +38067,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38227,7 +38227,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42825,7 +42825,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42985,7 +42985,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45069,7 +45069,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -49368,7 +49368,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -51441,7 +51441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52979,7 +52979,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56573,7 +56573,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -56992,7 +56992,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -61291,7 +61291,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -65589,7 +65589,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -69583,7 +69583,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71441,7 +71441,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75035,7 +75035,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -75454,7 +75454,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 25/05/2026 23:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 25/05/2026 23:53 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Historico: SEMANAS W17-W21, agregar W20 a arrays, W21 dinámico desde pickle
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9396,7 +9396,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12775,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16021,7 +16021,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16174,7 +16174,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16487,7 +16487,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19921,7 +19921,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -24220,7 +24220,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28519,7 +28519,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -30178,7 +30178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34277,7 +34277,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34696,7 +34696,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38989,7 +38989,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -39149,7 +39149,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43747,7 +43747,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43907,7 +43907,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45991,7 +45991,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50290,7 +50290,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52363,7 +52363,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -53902,7 +53902,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58001,7 +58001,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58420,7 +58420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -62719,7 +62719,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -67017,7 +67017,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71011,7 +71011,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -72870,7 +72870,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -76845,7 +76845,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77264,7 +77264,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 00:29 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cleanup: renders migrados a historico_module unificado, eliminar módulos obsoletos
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9396,7 +9396,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12775,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16021,7 +16021,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16174,7 +16174,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16487,7 +16487,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19921,7 +19921,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -24220,7 +24220,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28519,7 +28519,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -30178,7 +30178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34277,7 +34277,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34696,7 +34696,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38989,7 +38989,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -39149,7 +39149,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43747,7 +43747,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43907,7 +43907,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45991,7 +45991,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50290,7 +50290,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52363,7 +52363,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -53902,7 +53902,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58001,7 +58001,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58420,7 +58420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -62719,7 +62719,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -67017,7 +67017,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71011,7 +71011,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -72870,7 +72870,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -76845,7 +76845,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77264,7 +77264,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:08 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix histórico: eje X muestra las 5 semanas W17-W21 (no solo W17 y W21)
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9396,7 +9396,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12775,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16021,7 +16021,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16174,7 +16174,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16487,7 +16487,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19921,7 +19921,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -24220,7 +24220,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28519,7 +28519,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -30178,7 +30178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34277,7 +34277,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34696,7 +34696,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38989,7 +38989,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -39149,7 +39149,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43747,7 +43747,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43907,7 +43907,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45991,7 +45991,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50290,7 +50290,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52363,7 +52363,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -53902,7 +53902,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58001,7 +58001,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58420,7 +58420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -62719,7 +62719,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -67017,7 +67017,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71011,7 +71011,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -72870,7 +72870,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -76845,7 +76845,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77264,7 +77264,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 01:25 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix histórico: labels W17-W21 equiespaciados con position:absolute left:N%
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9396,7 +9396,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12775,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16021,7 +16021,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16174,7 +16174,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16487,7 +16487,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19921,7 +19921,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -24220,7 +24220,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28519,7 +28519,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -30178,7 +30178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34277,7 +34277,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34696,7 +34696,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38989,7 +38989,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -39149,7 +39149,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43747,7 +43747,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43907,7 +43907,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45991,7 +45991,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50290,7 +50290,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52363,7 +52363,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -53902,7 +53902,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58001,7 +58001,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58420,7 +58420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -62719,7 +62719,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -67017,7 +67017,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71011,7 +71011,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -72870,7 +72870,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -76845,7 +76845,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77264,7 +77264,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:28 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix histórico: spark bars normalizadas relativas al rango de la serie, fix val_actual*100
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9396,7 +9396,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12775,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16021,7 +16021,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16174,7 +16174,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16487,7 +16487,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19921,7 +19921,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -24220,7 +24220,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28519,7 +28519,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -30178,7 +30178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34277,7 +34277,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34696,7 +34696,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38989,7 +38989,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -39149,7 +39149,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43747,7 +43747,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43907,7 +43907,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45991,7 +45991,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50290,7 +50290,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52363,7 +52363,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -53902,7 +53902,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58001,7 +58001,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58420,7 +58420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -62719,7 +62719,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -67017,7 +67017,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71011,7 +71011,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -72870,7 +72870,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -76845,7 +76845,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77264,7 +77264,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix histórico: lineWidth=2px (curva no superficie), val_actual fracción→% correcto
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9396,7 +9396,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12775,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16021,7 +16021,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16174,7 +16174,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16487,7 +16487,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19921,7 +19921,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -24220,7 +24220,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28519,7 +28519,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -30178,7 +30178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34277,7 +34277,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34696,7 +34696,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38989,7 +38989,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -39149,7 +39149,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43747,7 +43747,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43907,7 +43907,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45991,7 +45991,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50290,7 +50290,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52363,7 +52363,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -53902,7 +53902,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58001,7 +58001,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58420,7 +58420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -62719,7 +62719,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -67017,7 +67017,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71011,7 +71011,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -72870,7 +72870,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -76845,7 +76845,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77264,7 +77264,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:45 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix histórico: CR accent #5C469C, area fill suave, puntos en color accent
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9396,7 +9396,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12775,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16021,7 +16021,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16174,7 +16174,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16487,7 +16487,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19921,7 +19921,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -24220,7 +24220,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28519,7 +28519,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -30178,7 +30178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34277,7 +34277,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34696,7 +34696,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38989,7 +38989,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -39149,7 +39149,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43747,7 +43747,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43907,7 +43907,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45991,7 +45991,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50290,7 +50290,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52363,7 +52363,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -53902,7 +53902,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58001,7 +58001,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58420,7 +58420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -62719,7 +62719,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -67017,7 +67017,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71011,7 +71011,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -72870,7 +72870,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -76845,7 +76845,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77264,7 +77264,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 02:52 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix gauge: Súper Crítica usa gris #8A8377 coherente con badge (como IPM Sin Conv)
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-21/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1757,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9396,7 +9396,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -12775,7 +12775,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16021,7 +16021,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16174,7 +16174,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16327,7 +16327,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -16487,7 +16487,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19921,7 +19921,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -24220,7 +24220,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28519,7 +28519,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -30178,7 +30178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34277,7 +34277,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34696,7 +34696,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38989,7 +38989,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -39149,7 +39149,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43747,7 +43747,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -43907,7 +43907,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -45991,7 +45991,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50290,7 +50290,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -52363,7 +52363,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -53902,7 +53902,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58001,7 +58001,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -58420,7 +58420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -62719,7 +62719,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -67017,7 +67017,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -71011,7 +71011,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -72870,7 +72870,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -76845,7 +76845,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77264,7 +77264,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 26/05/2026 03:05 · W20 · 12-18 may 2026</t>
+          <t>Generado: 26/05/2026 03:15 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>